<commit_message>
changing CSF-[brain] to only require 1 correlation value
</commit_message>
<xml_diff>
--- a/metabolomics_analysis/metabolites_analysis.xlsx
+++ b/metabolomics_analysis/metabolites_analysis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/laurenbell/Desktop/networks/metabolomics_analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{388EF5E5-A6DC-D740-9111-0364ADB5E06C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11A0B70C-3124-A74A-B5A0-9AE398584695}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="25800" windowHeight="15780" activeTab="5" xr2:uid="{11D052C1-3FE8-A645-8B41-A66CF54B9550}"/>
+    <workbookView xWindow="20" yWindow="500" windowWidth="28800" windowHeight="15780" activeTab="6" xr2:uid="{11D052C1-3FE8-A645-8B41-A66CF54B9550}"/>
   </bookViews>
   <sheets>
     <sheet name="External IDs" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="Duplicate Check FEC" sheetId="5" r:id="rId4"/>
     <sheet name="Duplicate Check CSF" sheetId="4" r:id="rId5"/>
     <sheet name="Marcello Comparison" sheetId="6" r:id="rId6"/>
+    <sheet name="Guiseppe + Marcello Comparison" sheetId="7" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'De-Derivatized Names'!$A$1:$C$67</definedName>
@@ -26,6 +27,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Duplicate Check FEC'!$A$1:$C$224</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Duplicate Check PLS'!$A$1:$C$375</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'External IDs'!$A$1:$F$935</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Guiseppe + Marcello Comparison'!$A$1:$J$67</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Marcello Comparison'!$A$1:$F$49</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -49,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4360" uniqueCount="1871">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4734" uniqueCount="2030">
   <si>
     <t>Pyrimidine, 5-methyl-2,4-bis[(trimethylsilyl)oxy]-</t>
   </si>
@@ -5662,13 +5664,490 @@
   </si>
   <si>
     <t>De_Derivatized</t>
+  </si>
+  <si>
+    <t>3-(Nona-4,7-dienoyl)oxirane-2-carboxamide</t>
+  </si>
+  <si>
+    <t>O=C(N)C1OC1C(=O)CC\C=C\C\C=C\C</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/5352018</t>
+  </si>
+  <si>
+    <t>NoName_52</t>
+  </si>
+  <si>
+    <t>Oc1nc(N)n(C)c1</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/26009888</t>
+  </si>
+  <si>
+    <t>OC(C=C=C(c1ccccc1)c1ccccc1)c1ccccc1</t>
+  </si>
+  <si>
+    <t>C#Cc1cc(ccc1)C#C</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/123130</t>
+  </si>
+  <si>
+    <t>2-Oxohexanoic Acid</t>
+  </si>
+  <si>
+    <t>CCCCC(=O)C(=O)O</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/159664</t>
+  </si>
+  <si>
+    <t>Cc1cccc(C)c1N=C1SCCCN1</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/5707</t>
+  </si>
+  <si>
+    <t>O=C(C)C(O)=C</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/13285096</t>
+  </si>
+  <si>
+    <t>Beta-Naphthoflavone</t>
+  </si>
+  <si>
+    <t>C1=CC=C(C=C1)C2=CC(=O)C3=C(O2)C=CC4=CC=CC=C43</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/Beta-Naphthoflavone</t>
+  </si>
+  <si>
+    <t>7Alpha-Hydroxycholesterol</t>
+  </si>
+  <si>
+    <t>C[C@H](CCCC(C)C)[C@H]1CC[C@@H]2[C@@]1(CC[C@H]3[C@H]2[C@@H](C=C4[C@@]3(CC[C@@H](C4)O)C)O)C</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/7alpha-Hydroxycholesterol</t>
+  </si>
+  <si>
+    <t>7-Amino-4-methylcoumarin</t>
+  </si>
+  <si>
+    <t>O=C1C=C(C)c2ccc(N)cc2O1</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/92249</t>
+  </si>
+  <si>
+    <t>2,2-Dihydroxyacetic acid</t>
+  </si>
+  <si>
+    <t>OC(=O)C(O)O</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/2723641</t>
+  </si>
+  <si>
+    <t>Glyceryl 2-acetate</t>
+  </si>
+  <si>
+    <t>O=C(C)OC(CO)CO</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/641349</t>
+  </si>
+  <si>
+    <t>Oc1ccc(CCN=Cc2c(F)c(F)c(F)c(F)c2F)cc1</t>
+  </si>
+  <si>
+    <t>OC1OC(CN2CCOCC2)C(O)C(O)C1O</t>
+  </si>
+  <si>
+    <t>beta-D-galactofuranose</t>
+  </si>
+  <si>
+    <t>O[C@H]1[C@H](O[C@@H](O)[C@@H]1O)C(O)CO</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/11019448</t>
+  </si>
+  <si>
+    <t>C#C</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/6326</t>
+  </si>
+  <si>
+    <t>O[C@H](CO)[C@H](O)\C=N/OC</t>
+  </si>
+  <si>
+    <t>3-Hydroxy-2-methylbutyric acid</t>
+  </si>
+  <si>
+    <t>OC(=O)C(C)C(O)C</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/160471</t>
+  </si>
+  <si>
+    <t>2,4-Dihydroxy-2-(hydroxymethyl)butanoic acid</t>
+  </si>
+  <si>
+    <t>OC(=O)C(O)(CO)CCO</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/86013822</t>
+  </si>
+  <si>
+    <t>4-(Hexadecylamino)benzoic acid</t>
+  </si>
+  <si>
+    <t>OC(=O)c1ccc(NCCCCCCCCCCCCCCCC)cc1</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/47263</t>
+  </si>
+  <si>
+    <t>O=C(O)C1CCC(O)CC1</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/151138</t>
+  </si>
+  <si>
+    <t>O=C(NCC(O)=O)c1ccc(O)cc1</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/151012</t>
+  </si>
+  <si>
+    <t>O[C@H]1[C@@H](O)[C@H](O)[C@@H](CO)O[C@@H]1N1CCOCC1</t>
+  </si>
+  <si>
+    <t>Hexanamide</t>
+  </si>
+  <si>
+    <t>O=C(N)CCCCC</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/12332</t>
+  </si>
+  <si>
+    <t>CC(C)CNC(=O)N1CCN=C1O</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/35699</t>
+  </si>
+  <si>
+    <t>Guanine</t>
+  </si>
+  <si>
+    <t>Nc1nc2[nH]cnc2c(O)n1</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/135398634</t>
+  </si>
+  <si>
+    <t>Carbamic Acid</t>
+  </si>
+  <si>
+    <t>OC(=O)N</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/277</t>
+  </si>
+  <si>
+    <t>2-Hydroxyglutaric acid</t>
+  </si>
+  <si>
+    <t>O=C(O)C(O)CCC(O)=O</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/43</t>
+  </si>
+  <si>
+    <t>O=C(O)CC(O)(C)CC(O)=O</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/1662</t>
+  </si>
+  <si>
+    <t>4-Hydroxypent-3-enoic acid</t>
+  </si>
+  <si>
+    <t>OC(=O)C\C=C(/O)C</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/6442606</t>
+  </si>
+  <si>
+    <t>Oc1nc(O)c(C)cn1</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/1135</t>
+  </si>
+  <si>
+    <t>Nc1c2ccccc2nc2CCCCc12</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/1935</t>
+  </si>
+  <si>
+    <t>CN1C(=O)N(C)C(CO)=C(C)C1=O</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/129651811</t>
+  </si>
+  <si>
+    <t>O=C1NC(Cc2ccccc2)C(=O)NC1CC(=O)O</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/119494</t>
+  </si>
+  <si>
+    <t>3-Mercaptopropionic Acid</t>
+  </si>
+  <si>
+    <t>SCCC(=O)O</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/6514</t>
+  </si>
+  <si>
+    <t>Oct-2-enoic acid</t>
+  </si>
+  <si>
+    <t>O=C(O)C=CCCCCC</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/73850</t>
+  </si>
+  <si>
+    <t>5-Ethyl-2-indolecarboxylic acid</t>
+  </si>
+  <si>
+    <t>OC(=O)c1cc2cc(ccc2[nH]1)CC</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/269697</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/14345506</t>
+  </si>
+  <si>
+    <t>CCOC(=O)N1N(CC(O)=C2CCCCC12)C(=O)OCC</t>
+  </si>
+  <si>
+    <t>O\C(=C/C(CC)c1ccccc1)\c1ccccc1</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/20606316</t>
+  </si>
+  <si>
+    <t>O=C(C)OC(C)C(O)C</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/143344</t>
+  </si>
+  <si>
+    <t>Phenolphthalein</t>
+  </si>
+  <si>
+    <t>O=C1OC(c2ccccc12)(c1ccc(O)cc1)c1ccc(O)cc1</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/4764</t>
+  </si>
+  <si>
+    <t>2-Ethyl-1,3-butanediol</t>
+  </si>
+  <si>
+    <t>OC(C)C(CO)CC</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/47955</t>
+  </si>
+  <si>
+    <t>3-Amino-9-ethylcarbazole</t>
+  </si>
+  <si>
+    <t>Nc1cc2c(cc1)n(CC)c1ccccc12</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/8588</t>
+  </si>
+  <si>
+    <t>CNC(C)C(O)c1ccc(O)cc1</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/9701</t>
+  </si>
+  <si>
+    <t>OC(=O)[C@@H](N)CCCC</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/21236</t>
+  </si>
+  <si>
+    <t>3,14-Dihydroxy-17-methyl-4,5-epoxymorphinan-6-one</t>
+  </si>
+  <si>
+    <t>OC12CCC(=O)C3Oc4c5c(CC1N(C)CCC352)ccc4O</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/4639</t>
+  </si>
+  <si>
+    <t>O=C(O)C1CCCN1C(O)=O</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/14794868</t>
+  </si>
+  <si>
+    <t>Cc1cn[nH]c1</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/3406</t>
+  </si>
+  <si>
+    <t>Dimethylhydantoin</t>
+  </si>
+  <si>
+    <t>OC1=NC(C)(C)C(O)=N1</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/6491</t>
+  </si>
+  <si>
+    <t>3-hydroxybut-2-enoic acid</t>
+  </si>
+  <si>
+    <t>OC(=O)\C=C(\O)C</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/54715757</t>
+  </si>
+  <si>
+    <t>2-Methylcyclohexylamine, tert-butyldimethylsilyl ether</t>
+  </si>
+  <si>
+    <t>CC1CCCCC1N</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/23432</t>
+  </si>
+  <si>
+    <t>O=C(C)OCCC1(CO1)CO</t>
+  </si>
+  <si>
+    <t>COc1cc(C=O)cc(OC)c1O</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/8655</t>
+  </si>
+  <si>
+    <t>OCC1(COCOC1)CC</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/78860</t>
+  </si>
+  <si>
+    <t>Nonan-5-ol</t>
+  </si>
+  <si>
+    <t>CCCCC(CCCC)O</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/12202</t>
+  </si>
+  <si>
+    <t>6-Aminohexanoic Acid</t>
+  </si>
+  <si>
+    <t>C(CCC(=O)O)CCN</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/564</t>
+  </si>
+  <si>
+    <t>Oc1nc(N)ccn1</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/597</t>
+  </si>
+  <si>
+    <t>Glycine methyl ester</t>
+  </si>
+  <si>
+    <t>O=C(OC)CN</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/69221</t>
+  </si>
+  <si>
+    <t>Hymexazol</t>
+  </si>
+  <si>
+    <t>Oc1noc(C)c1</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/24781</t>
+  </si>
+  <si>
+    <t>Kojic Acid</t>
+  </si>
+  <si>
+    <t>C1=C(OC=C(C1=O)O)CO</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/3840</t>
+  </si>
+  <si>
+    <t>N[C@@H](Cc1nc[nH]c1)C(O)=O</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/6274</t>
+  </si>
+  <si>
+    <t>OC(=O)C(C)CO</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/87</t>
+  </si>
+  <si>
+    <t>Propionic Acid</t>
+  </si>
+  <si>
+    <t>OC(=O)CC</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/1032</t>
+  </si>
+  <si>
+    <t>OC(=O)/C(O)=C/CCC</t>
+  </si>
+  <si>
+    <t>https://pubchem.ncbi.nlm.nih.gov/compound/69980390</t>
+  </si>
+  <si>
+    <t>Un-derivatized name</t>
+  </si>
+  <si>
+    <t>Smile</t>
+  </si>
+  <si>
+    <t>link</t>
+  </si>
+  <si>
+    <t>Guiseppe ID</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -5709,8 +6188,43 @@
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Aptos Display"/>
+      <family val="2"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Aptos Display"/>
+      <family val="2"/>
+      <scheme val="major"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -5759,6 +6273,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -5778,10 +6298,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -5804,11 +6325,90 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="8">
+  <dxfs count="14">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -5856,14 +6456,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -23621,10 +24213,10 @@
     </sortState>
   </autoFilter>
   <conditionalFormatting sqref="D1:F1 C1:C1048576">
-    <cfRule type="cellIs" dxfId="4" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="11" priority="1" operator="equal">
       <formula>FALSE</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="2" operator="equal">
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
@@ -23653,7 +24245,7 @@
         <v>1788</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>14</v>
       </c>
@@ -23664,7 +24256,7 @@
         <v>91696873</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>15</v>
       </c>
@@ -23675,7 +24267,7 @@
         <v>91706643</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>8</v>
       </c>
@@ -23686,7 +24278,7 @@
         <v>601546</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>2</v>
       </c>
@@ -23697,7 +24289,7 @@
         <v>142239</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>21</v>
       </c>
@@ -23705,7 +24297,7 @@
         <v>1791</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>19</v>
       </c>
@@ -23716,7 +24308,7 @@
         <v>91740490</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>7</v>
       </c>
@@ -23727,7 +24319,7 @@
         <v>588565</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
         <v>22</v>
       </c>
@@ -23735,7 +24327,7 @@
         <v>1793</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>23</v>
       </c>
@@ -23743,7 +24335,7 @@
         <v>1794</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>18</v>
       </c>
@@ -23754,7 +24346,7 @@
         <v>91736840</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
         <v>24</v>
       </c>
@@ -23762,7 +24354,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
         <v>13</v>
       </c>
@@ -23773,7 +24365,7 @@
         <v>91696644</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
         <v>9</v>
       </c>
@@ -23784,7 +24376,7 @@
         <v>601551</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
         <v>25</v>
       </c>
@@ -23792,7 +24384,7 @@
         <v>1796</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>26</v>
       </c>
@@ -23800,7 +24392,7 @@
         <v>1797</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
         <v>1</v>
       </c>
@@ -23811,7 +24403,7 @@
         <v>84564</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
         <v>27</v>
       </c>
@@ -23819,7 +24411,7 @@
         <v>1766</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>28</v>
       </c>
@@ -23827,7 +24419,7 @@
         <v>1798</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
         <v>29</v>
       </c>
@@ -23835,7 +24427,7 @@
         <v>1799</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
         <v>20</v>
       </c>
@@ -23846,7 +24438,7 @@
         <v>91741325</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
         <v>4</v>
       </c>
@@ -23857,7 +24449,7 @@
         <v>533404</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
         <v>30</v>
       </c>
@@ -23865,7 +24457,7 @@
         <v>1801</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
         <v>31</v>
       </c>
@@ -23873,7 +24465,7 @@
         <v>1768</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
         <v>12</v>
       </c>
@@ -23884,7 +24476,7 @@
         <v>18935209</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
         <v>16</v>
       </c>
@@ -23895,7 +24487,7 @@
         <v>91729087</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
         <v>3</v>
       </c>
@@ -23906,7 +24498,7 @@
         <v>530172</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
         <v>11</v>
       </c>
@@ -23917,7 +24509,7 @@
         <v>3015764</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
         <v>32</v>
       </c>
@@ -23925,7 +24517,7 @@
         <v>1804</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
         <v>33</v>
       </c>
@@ -23933,7 +24525,7 @@
         <v>1805</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
         <v>34</v>
       </c>
@@ -23941,7 +24533,7 @@
         <v>1806</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
         <v>0</v>
       </c>
@@ -23952,7 +24544,7 @@
         <v>81705</v>
       </c>
     </row>
-    <row r="33" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="4" t="s">
         <v>35</v>
       </c>
@@ -23960,7 +24552,7 @@
         <v>1771</v>
       </c>
     </row>
-    <row r="34" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
         <v>6</v>
       </c>
@@ -23971,7 +24563,7 @@
         <v>553578</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
         <v>17</v>
       </c>
@@ -23982,7 +24574,7 @@
         <v>91733438</v>
       </c>
     </row>
-    <row r="36" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
         <v>10</v>
       </c>
@@ -23993,7 +24585,7 @@
         <v>637748</v>
       </c>
     </row>
-    <row r="37" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" s="4" t="s">
         <v>5</v>
       </c>
@@ -24004,7 +24596,7 @@
         <v>533405</v>
       </c>
     </row>
-    <row r="38" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
         <v>17</v>
       </c>
@@ -24015,7 +24607,7 @@
         <v>91733438</v>
       </c>
     </row>
-    <row r="39" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
         <v>36</v>
       </c>
@@ -24023,7 +24615,7 @@
         <v>1810</v>
       </c>
     </row>
-    <row r="40" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="A40" s="6" t="s">
         <v>540</v>
       </c>
@@ -24034,7 +24626,7 @@
         <v>91742919</v>
       </c>
     </row>
-    <row r="41" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" s="6" t="s">
         <v>546</v>
       </c>
@@ -24045,7 +24637,7 @@
         <v>14345506</v>
       </c>
     </row>
-    <row r="42" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="A42" s="6" t="s">
         <v>549</v>
       </c>
@@ -24056,7 +24648,7 @@
         <v>91716313</v>
       </c>
     </row>
-    <row r="43" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="6" t="s">
         <v>553</v>
       </c>
@@ -24067,7 +24659,7 @@
         <v>553703</v>
       </c>
     </row>
-    <row r="44" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" s="6" t="s">
         <v>563</v>
       </c>
@@ -24078,7 +24670,7 @@
         <v>5378122</v>
       </c>
     </row>
-    <row r="45" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="6" t="s">
         <v>569</v>
       </c>
@@ -24089,7 +24681,7 @@
         <v>575921</v>
       </c>
     </row>
-    <row r="46" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="A46" s="6" t="s">
         <v>577</v>
       </c>
@@ -24100,7 +24692,7 @@
         <v>91741551</v>
       </c>
     </row>
-    <row r="47" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="A47" s="6" t="s">
         <v>586</v>
       </c>
@@ -24108,7 +24700,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="48" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="A48" s="6" t="s">
         <v>602</v>
       </c>
@@ -24116,7 +24708,7 @@
         <v>1815</v>
       </c>
     </row>
-    <row r="49" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="A49" s="6" t="s">
         <v>604</v>
       </c>
@@ -24127,7 +24719,7 @@
         <v>554546</v>
       </c>
     </row>
-    <row r="50" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="6" t="s">
         <v>612</v>
       </c>
@@ -24138,7 +24730,7 @@
         <v>91697039</v>
       </c>
     </row>
-    <row r="51" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="A51" s="6" t="s">
         <v>616</v>
       </c>
@@ -24149,7 +24741,7 @@
         <v>10357235</v>
       </c>
     </row>
-    <row r="52" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" s="6" t="s">
         <v>622</v>
       </c>
@@ -24160,7 +24752,7 @@
         <v>575923</v>
       </c>
     </row>
-    <row r="53" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="A53" s="6" t="s">
         <v>638</v>
       </c>
@@ -24171,7 +24763,7 @@
         <v>91697308</v>
       </c>
     </row>
-    <row r="54" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="A54" s="6" t="s">
         <v>642</v>
       </c>
@@ -24179,7 +24771,7 @@
         <v>1775</v>
       </c>
     </row>
-    <row r="55" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="A55" s="6" t="s">
         <v>643</v>
       </c>
@@ -24187,7 +24779,7 @@
         <v>1776</v>
       </c>
     </row>
-    <row r="56" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" s="6" t="s">
         <v>653</v>
       </c>
@@ -24198,7 +24790,7 @@
         <v>91740788</v>
       </c>
     </row>
-    <row r="57" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="A57" s="6" t="s">
         <v>687</v>
       </c>
@@ -24206,7 +24798,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="58" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="A58" s="6" t="s">
         <v>700</v>
       </c>
@@ -24214,7 +24806,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="59" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="A59" s="6" t="s">
         <v>706</v>
       </c>
@@ -24225,7 +24817,7 @@
         <v>19104051</v>
       </c>
     </row>
-    <row r="60" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="A60" s="6" t="s">
         <v>713</v>
       </c>
@@ -24233,7 +24825,7 @@
         <v>1778</v>
       </c>
     </row>
-    <row r="61" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="A61" s="6" t="s">
         <v>718</v>
       </c>
@@ -24241,7 +24833,7 @@
         <v>1779</v>
       </c>
     </row>
-    <row r="62" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" s="6" t="s">
         <v>743</v>
       </c>
@@ -24252,7 +24844,7 @@
         <v>91693841</v>
       </c>
     </row>
-    <row r="63" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" s="6" t="s">
         <v>746</v>
       </c>
@@ -24260,7 +24852,7 @@
         <v>1780</v>
       </c>
     </row>
-    <row r="64" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" s="6" t="s">
         <v>754</v>
       </c>
@@ -24271,7 +24863,7 @@
         <v>91697075</v>
       </c>
     </row>
-    <row r="65" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="A65" s="6" t="s">
         <v>765</v>
       </c>
@@ -24279,7 +24871,7 @@
         <v>1820</v>
       </c>
     </row>
-    <row r="66" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="A66" s="6" t="s">
         <v>766</v>
       </c>
@@ -24287,7 +24879,7 @@
         <v>767</v>
       </c>
     </row>
-    <row r="67" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="A67" s="6" t="s">
         <v>780</v>
       </c>
@@ -24302,7 +24894,7 @@
   <autoFilter ref="A1:C67" xr:uid="{F74EA60A-F317-264B-8424-78A87D50A412}">
     <filterColumn colId="0">
       <customFilters>
-        <customFilter val="*trimethylsilyl*"/>
+        <customFilter operator="notEqual" val="*trimethylsilyl*"/>
       </customFilters>
     </filterColumn>
   </autoFilter>
@@ -29971,11 +30563,11 @@
   </sheetData>
   <autoFilter ref="A1:C375" xr:uid="{4188BBC8-34B5-FB4F-9E6B-EBFEE61392C2}">
     <filterColumn colId="1">
-      <colorFilter dxfId="6"/>
+      <colorFilter dxfId="13"/>
     </filterColumn>
   </autoFilter>
   <conditionalFormatting sqref="B1:B1048576">
-    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -32334,11 +32926,11 @@
   </sheetData>
   <autoFilter ref="A1:C224" xr:uid="{28BCC6CD-92FE-2549-8CF0-B350441AC06D}">
     <filterColumn colId="1">
-      <colorFilter dxfId="7"/>
+      <colorFilter dxfId="12"/>
     </filterColumn>
   </autoFilter>
   <conditionalFormatting sqref="B1:B1048576">
-    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -33123,7 +33715,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" s="3" t="s">
         <v>608</v>
       </c>
@@ -34610,7 +35202,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="213" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A213" s="3" t="s">
         <v>288</v>
       </c>
@@ -34643,7 +35235,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="216" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A216" s="3" t="s">
         <v>723</v>
       </c>
@@ -35044,7 +35636,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="253" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A253" s="3" t="s">
         <v>749</v>
       </c>
@@ -35434,7 +36026,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="289" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A289" s="3" t="s">
         <v>358</v>
       </c>
@@ -35919,10 +36511,10 @@
     </row>
     <row r="334" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="A334" s="3" t="s">
-        <v>1780</v>
+        <v>767</v>
       </c>
       <c r="B334">
-        <v>21236</v>
+        <v>1032</v>
       </c>
       <c r="C334" t="b">
         <v>1</v>
@@ -35950,12 +36542,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="337" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:3" ht="18" hidden="1" x14ac:dyDescent="0.25">
       <c r="A337" s="3" t="s">
-        <v>767</v>
+        <v>1780</v>
       </c>
       <c r="B337">
-        <v>1032</v>
+        <v>21236</v>
       </c>
       <c r="C337" t="b">
         <v>1</v>
@@ -35971,12 +36563,15 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:C338" xr:uid="{10886208-4343-B54A-9C3F-CEF32D0EA18E}">
-    <filterColumn colId="1">
-      <colorFilter dxfId="5"/>
+    <filterColumn colId="0">
+      <colorFilter dxfId="0"/>
     </filterColumn>
   </autoFilter>
   <conditionalFormatting sqref="B1:B1048576">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A1:A1048576">
+    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -35984,7 +36579,6 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4FC2FD3-2DF4-BF4A-B499-41C8A1E04B96}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:F49"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
@@ -36034,7 +36628,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>15</v>
       </c>
@@ -36055,7 +36649,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>8</v>
       </c>
@@ -36072,7 +36666,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>2</v>
       </c>
@@ -36093,7 +36687,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>21</v>
       </c>
@@ -36129,7 +36723,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>7</v>
       </c>
@@ -36150,7 +36744,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
         <v>22</v>
       </c>
@@ -36186,7 +36780,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>18</v>
       </c>
@@ -36207,7 +36801,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
         <v>24</v>
       </c>
@@ -36228,7 +36822,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
         <v>13</v>
       </c>
@@ -36268,7 +36862,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
         <v>25</v>
       </c>
@@ -36304,7 +36898,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
         <v>1</v>
       </c>
@@ -36365,7 +36959,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
         <v>29</v>
       </c>
@@ -36386,7 +36980,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
         <v>20</v>
       </c>
@@ -36407,7 +37001,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
         <v>4</v>
       </c>
@@ -36428,7 +37022,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
         <v>30</v>
       </c>
@@ -36449,7 +37043,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:6" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
         <v>31</v>
       </c>
@@ -36466,7 +37060,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:6" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
         <v>12</v>
       </c>
@@ -36506,7 +37100,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
         <v>3</v>
       </c>
@@ -36548,7 +37142,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
         <v>32</v>
       </c>
@@ -36569,7 +37163,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:6" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
         <v>33</v>
       </c>
@@ -36611,7 +37205,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:6" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
         <v>0</v>
       </c>
@@ -36632,7 +37226,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:6" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A33" s="4" t="s">
         <v>35</v>
       </c>
@@ -36653,7 +37247,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:6" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
         <v>6</v>
       </c>
@@ -36670,7 +37264,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:6" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
         <v>17</v>
       </c>
@@ -36691,7 +37285,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:6" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
         <v>10</v>
       </c>
@@ -36733,7 +37327,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:6" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
         <v>17</v>
       </c>
@@ -36754,7 +37348,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:6" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
         <v>36</v>
       </c>
@@ -36794,7 +37388,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:6" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A41" s="6" t="s">
         <v>553</v>
       </c>
@@ -36811,7 +37405,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:6" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A42" s="6" t="s">
         <v>563</v>
       </c>
@@ -36828,7 +37422,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:6" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A43" s="6" t="s">
         <v>569</v>
       </c>
@@ -36849,7 +37443,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:6" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A44" s="6" t="s">
         <v>612</v>
       </c>
@@ -36889,7 +37483,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:6" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A46" s="6" t="s">
         <v>653</v>
       </c>
@@ -36929,7 +37523,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:6" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A48" s="6" t="s">
         <v>746</v>
       </c>
@@ -36950,7 +37544,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:6" ht="18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A49" s="6" t="s">
         <v>754</v>
       </c>
@@ -36972,13 +37566,2097 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F49" xr:uid="{E4FC2FD3-2DF4-BF4A-B499-41C8A1E04B96}">
-    <filterColumn colId="5">
+  <autoFilter ref="A1:F49" xr:uid="{E4FC2FD3-2DF4-BF4A-B499-41C8A1E04B96}"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2442BCC8-4903-A242-813F-023B53DEA0F4}">
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:J67"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="87.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="60.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="69.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="53.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.6640625" customWidth="1"/>
+    <col min="8" max="8" width="61.5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" ht="19" x14ac:dyDescent="0.25">
+      <c r="A1" s="11" t="s">
+        <v>1861</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>1862</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>1864</v>
+      </c>
+      <c r="D1" s="11" t="s">
+        <v>1863</v>
+      </c>
+      <c r="E1" s="11" t="s">
+        <v>1865</v>
+      </c>
+      <c r="F1" s="27" t="s">
+        <v>2026</v>
+      </c>
+      <c r="G1" s="27" t="s">
+        <v>2027</v>
+      </c>
+      <c r="H1" s="27" t="s">
+        <v>2028</v>
+      </c>
+      <c r="I1" s="27" t="s">
+        <v>2029</v>
+      </c>
+      <c r="J1" s="27" t="s">
+        <v>1867</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="20" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="21" t="s">
+        <v>1821</v>
+      </c>
+      <c r="C2" s="22"/>
+      <c r="D2" s="20" t="s">
+        <v>1761</v>
+      </c>
+      <c r="E2" s="22">
+        <v>5352018</v>
+      </c>
+      <c r="F2" s="23" t="s">
+        <v>1871</v>
+      </c>
+      <c r="G2" t="s">
+        <v>1872</v>
+      </c>
+      <c r="H2" s="24" t="s">
+        <v>1873</v>
+      </c>
+      <c r="I2">
+        <v>5352018</v>
+      </c>
+      <c r="J2" t="b">
+        <f>IF(I2=E2, TRUE, FALSE)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="21" t="s">
+        <v>1789</v>
+      </c>
+      <c r="C3" s="22">
+        <v>26009888</v>
+      </c>
+      <c r="D3" s="20" t="s">
+        <v>1789</v>
+      </c>
+      <c r="E3" s="22">
+        <v>26009888</v>
+      </c>
+      <c r="F3" t="s">
+        <v>1874</v>
+      </c>
+      <c r="G3" t="s">
+        <v>1875</v>
+      </c>
+      <c r="H3" s="24" t="s">
+        <v>1876</v>
+      </c>
+      <c r="I3">
+        <v>26009888</v>
+      </c>
+      <c r="J3" t="b">
+        <f t="shared" ref="J3:J49" si="0">IF(I3=E3, TRUE, FALSE)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="20" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="21" t="s">
+        <v>1822</v>
+      </c>
+      <c r="C4" s="22"/>
+      <c r="D4" s="20" t="s">
+        <v>1762</v>
+      </c>
+      <c r="E4" s="22"/>
+      <c r="G4" t="s">
+        <v>1877</v>
+      </c>
+      <c r="J4" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="20" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="21" t="s">
+        <v>1823</v>
+      </c>
+      <c r="C5" s="22">
+        <v>123130</v>
+      </c>
+      <c r="D5" s="20" t="s">
+        <v>1790</v>
+      </c>
+      <c r="E5" s="22">
+        <v>123130</v>
+      </c>
+      <c r="F5" t="s">
+        <v>1790</v>
+      </c>
+      <c r="G5" t="s">
+        <v>1878</v>
+      </c>
+      <c r="H5" s="24" t="s">
+        <v>1879</v>
+      </c>
+      <c r="I5">
+        <v>123130</v>
+      </c>
+      <c r="J5" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A6" s="20" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" s="21" t="s">
+        <v>1824</v>
+      </c>
+      <c r="C6" s="22"/>
+      <c r="D6" s="20" t="s">
+        <v>1791</v>
+      </c>
+      <c r="E6" s="22"/>
+      <c r="F6" t="s">
+        <v>1880</v>
+      </c>
+      <c r="G6" t="s">
+        <v>1881</v>
+      </c>
+      <c r="H6" s="24" t="s">
+        <v>1882</v>
+      </c>
+      <c r="I6">
+        <v>159664</v>
+      </c>
+      <c r="J6" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="21" t="s">
+        <v>1825</v>
+      </c>
+      <c r="C7" s="22"/>
+      <c r="D7" s="20" t="s">
+        <v>373</v>
+      </c>
+      <c r="E7" s="22">
+        <v>5707</v>
+      </c>
+      <c r="F7" t="s">
+        <v>373</v>
+      </c>
+      <c r="G7" t="s">
+        <v>1883</v>
+      </c>
+      <c r="H7" s="24" t="s">
+        <v>1884</v>
+      </c>
+      <c r="I7">
+        <v>5707</v>
+      </c>
+      <c r="J7" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="20" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="21" t="s">
+        <v>1826</v>
+      </c>
+      <c r="C8" s="22">
+        <v>13285096</v>
+      </c>
+      <c r="D8" s="20" t="s">
+        <v>1792</v>
+      </c>
+      <c r="E8" s="22">
+        <v>13285096</v>
+      </c>
+      <c r="F8" t="s">
+        <v>1792</v>
+      </c>
+      <c r="G8" t="s">
+        <v>1885</v>
+      </c>
+      <c r="H8" s="24" t="s">
+        <v>1886</v>
+      </c>
+      <c r="I8">
+        <v>13285096</v>
+      </c>
+      <c r="J8" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A9" s="20" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" s="21" t="s">
+        <v>1827</v>
+      </c>
+      <c r="C9" s="22"/>
+      <c r="D9" s="20" t="s">
+        <v>1793</v>
+      </c>
+      <c r="E9" s="22"/>
+      <c r="F9" t="s">
+        <v>1887</v>
+      </c>
+      <c r="G9" s="25" t="s">
+        <v>1888</v>
+      </c>
+      <c r="H9" s="24" t="s">
+        <v>1889</v>
+      </c>
+      <c r="I9">
+        <v>2361</v>
+      </c>
+      <c r="J9" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="B10" s="21" t="s">
+        <v>1828</v>
+      </c>
+      <c r="C10" s="22"/>
+      <c r="D10" s="20" t="s">
+        <v>1794</v>
+      </c>
+      <c r="E10" s="22">
+        <v>107722</v>
+      </c>
+      <c r="F10" t="s">
+        <v>1890</v>
+      </c>
+      <c r="G10" t="s">
+        <v>1891</v>
+      </c>
+      <c r="H10" s="24" t="s">
+        <v>1892</v>
+      </c>
+      <c r="I10">
+        <v>107722</v>
+      </c>
+      <c r="J10" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" s="21" t="s">
+        <v>1763</v>
+      </c>
+      <c r="C11" s="22">
+        <v>92249</v>
+      </c>
+      <c r="D11" s="20" t="s">
+        <v>1763</v>
+      </c>
+      <c r="E11" s="22">
+        <v>92249</v>
+      </c>
+      <c r="F11" t="s">
+        <v>1893</v>
+      </c>
+      <c r="G11" t="s">
+        <v>1894</v>
+      </c>
+      <c r="H11" s="24" t="s">
+        <v>1895</v>
+      </c>
+      <c r="I11">
+        <v>92249</v>
+      </c>
+      <c r="J11" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A12" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="B12" s="21" t="s">
+        <v>1829</v>
+      </c>
+      <c r="C12" s="22">
+        <v>757</v>
+      </c>
+      <c r="D12" s="20" t="s">
+        <v>258</v>
+      </c>
+      <c r="E12" s="22">
+        <v>757</v>
+      </c>
+      <c r="F12" t="s">
+        <v>1896</v>
+      </c>
+      <c r="G12" t="s">
+        <v>1897</v>
+      </c>
+      <c r="H12" s="24" t="s">
+        <v>1898</v>
+      </c>
+      <c r="I12">
+        <v>2723641</v>
+      </c>
+      <c r="J12" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A13" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13" s="21" t="s">
+        <v>1830</v>
+      </c>
+      <c r="C13" s="22">
+        <v>33510</v>
+      </c>
+      <c r="D13" s="20" t="s">
+        <v>1764</v>
+      </c>
+      <c r="E13" s="22">
+        <v>33510</v>
+      </c>
+      <c r="F13" t="s">
+        <v>1899</v>
+      </c>
+      <c r="G13" t="s">
+        <v>1900</v>
+      </c>
+      <c r="H13" s="24" t="s">
+        <v>1901</v>
+      </c>
+      <c r="I13">
+        <v>641349</v>
+      </c>
+      <c r="J13" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="B14" s="21" t="s">
+        <v>1831</v>
+      </c>
+      <c r="C14" s="22">
+        <v>5610</v>
+      </c>
+      <c r="D14" s="20" t="s">
+        <v>1795</v>
+      </c>
+      <c r="E14" s="22"/>
+      <c r="G14" t="s">
+        <v>1902</v>
+      </c>
+      <c r="J14" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="20" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15" s="21" t="s">
+        <v>1832</v>
+      </c>
+      <c r="C15" s="22"/>
+      <c r="D15" s="20" t="s">
+        <v>1796</v>
+      </c>
+      <c r="E15" s="22"/>
+      <c r="G15" t="s">
+        <v>1903</v>
+      </c>
+      <c r="J15" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A16" s="20" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16" s="21" t="s">
+        <v>1833</v>
+      </c>
+      <c r="C16" s="22">
+        <v>6036</v>
+      </c>
+      <c r="D16" s="20" t="s">
+        <v>1797</v>
+      </c>
+      <c r="E16" s="22"/>
+      <c r="F16" t="s">
+        <v>1904</v>
+      </c>
+      <c r="G16" t="s">
+        <v>1905</v>
+      </c>
+      <c r="H16" s="24" t="s">
+        <v>1906</v>
+      </c>
+      <c r="I16">
+        <v>11019448</v>
+      </c>
+      <c r="J16" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="20" t="s">
+        <v>1</v>
+      </c>
+      <c r="B17" s="21" t="s">
+        <v>1834</v>
+      </c>
+      <c r="C17" s="22">
+        <v>6326</v>
+      </c>
+      <c r="D17" s="20" t="s">
+        <v>1765</v>
+      </c>
+      <c r="E17" s="22">
+        <v>6326</v>
+      </c>
+      <c r="F17" t="s">
+        <v>1765</v>
+      </c>
+      <c r="G17" t="s">
+        <v>1907</v>
+      </c>
+      <c r="H17" s="24" t="s">
+        <v>1908</v>
+      </c>
+      <c r="I17">
+        <v>6326</v>
+      </c>
+      <c r="J17" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="B18" s="21" t="s">
+        <v>1835</v>
+      </c>
+      <c r="C18" s="22">
+        <v>94176</v>
+      </c>
+      <c r="D18" s="20" t="s">
+        <v>1766</v>
+      </c>
+      <c r="E18" s="22"/>
+      <c r="G18" t="s">
+        <v>1909</v>
+      </c>
+      <c r="J18" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A19" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="B19" s="21" t="s">
+        <v>1836</v>
+      </c>
+      <c r="C19" s="22">
+        <v>160471</v>
+      </c>
+      <c r="D19" s="20" t="s">
+        <v>1798</v>
+      </c>
+      <c r="E19" s="22">
+        <v>95433</v>
+      </c>
+      <c r="F19" t="s">
+        <v>1910</v>
+      </c>
+      <c r="G19" t="s">
+        <v>1911</v>
+      </c>
+      <c r="H19" s="24" t="s">
+        <v>1912</v>
+      </c>
+      <c r="I19">
+        <v>160471</v>
+      </c>
+      <c r="J19" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A20" s="20" t="s">
+        <v>29</v>
+      </c>
+      <c r="B20" s="21" t="s">
+        <v>1837</v>
+      </c>
+      <c r="C20" s="22">
+        <v>192742</v>
+      </c>
+      <c r="D20" s="20" t="s">
+        <v>1799</v>
+      </c>
+      <c r="E20" s="22">
+        <v>192742</v>
+      </c>
+      <c r="F20" t="s">
+        <v>1913</v>
+      </c>
+      <c r="G20" t="s">
+        <v>1914</v>
+      </c>
+      <c r="H20" s="24" t="s">
+        <v>1915</v>
+      </c>
+      <c r="I20">
+        <v>86013822</v>
+      </c>
+      <c r="J20" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" s="21" t="s">
+        <v>1767</v>
+      </c>
+      <c r="C21" s="22">
+        <v>47263</v>
+      </c>
+      <c r="D21" s="20" t="s">
+        <v>1767</v>
+      </c>
+      <c r="E21" s="22">
+        <v>47263</v>
+      </c>
+      <c r="F21" t="s">
+        <v>1916</v>
+      </c>
+      <c r="G21" t="s">
+        <v>1917</v>
+      </c>
+      <c r="H21" s="24" t="s">
+        <v>1918</v>
+      </c>
+      <c r="I21">
+        <v>47263</v>
+      </c>
+      <c r="J21" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="20" t="s">
+        <v>4</v>
+      </c>
+      <c r="B22" s="21" t="s">
+        <v>1838</v>
+      </c>
+      <c r="C22" s="22">
+        <v>151138</v>
+      </c>
+      <c r="D22" s="20" t="s">
+        <v>1800</v>
+      </c>
+      <c r="E22" s="22">
+        <v>151138</v>
+      </c>
+      <c r="F22" t="s">
+        <v>1800</v>
+      </c>
+      <c r="G22" t="s">
+        <v>1919</v>
+      </c>
+      <c r="H22" s="24" t="s">
+        <v>1920</v>
+      </c>
+      <c r="I22">
+        <v>151138</v>
+      </c>
+      <c r="J22" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="B23" s="21" t="s">
+        <v>1839</v>
+      </c>
+      <c r="C23" s="22">
+        <v>151012</v>
+      </c>
+      <c r="D23" s="20" t="s">
+        <v>1801</v>
+      </c>
+      <c r="E23" s="22">
+        <v>151012</v>
+      </c>
+      <c r="F23" t="s">
+        <v>1801</v>
+      </c>
+      <c r="G23" t="s">
+        <v>1921</v>
+      </c>
+      <c r="H23" s="24" t="s">
+        <v>1922</v>
+      </c>
+      <c r="I23">
+        <v>151012</v>
+      </c>
+      <c r="J23" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="B24" s="21" t="s">
+        <v>1840</v>
+      </c>
+      <c r="C24" s="22"/>
+      <c r="D24" s="20" t="s">
+        <v>1768</v>
+      </c>
+      <c r="E24" s="22"/>
+      <c r="G24" t="s">
+        <v>1923</v>
+      </c>
+      <c r="J24" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="B25" s="21" t="s">
+        <v>1841</v>
+      </c>
+      <c r="C25" s="22">
+        <v>12332</v>
+      </c>
+      <c r="D25" s="20" t="s">
+        <v>1769</v>
+      </c>
+      <c r="E25" s="22">
+        <v>12332</v>
+      </c>
+      <c r="F25" t="s">
+        <v>1924</v>
+      </c>
+      <c r="G25" t="s">
+        <v>1925</v>
+      </c>
+      <c r="H25" s="24" t="s">
+        <v>1926</v>
+      </c>
+      <c r="I25">
+        <v>12332</v>
+      </c>
+      <c r="J25" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="20" t="s">
+        <v>16</v>
+      </c>
+      <c r="B26" s="21" t="s">
+        <v>1842</v>
+      </c>
+      <c r="C26" s="22"/>
+      <c r="D26" s="20" t="s">
+        <v>1802</v>
+      </c>
+      <c r="E26" s="22">
+        <v>35699</v>
+      </c>
+      <c r="F26" t="s">
+        <v>1802</v>
+      </c>
+      <c r="G26" t="s">
+        <v>1927</v>
+      </c>
+      <c r="H26" s="24" t="s">
+        <v>1928</v>
+      </c>
+      <c r="I26">
+        <v>35699</v>
+      </c>
+      <c r="J26" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="B27" s="21" t="s">
+        <v>1803</v>
+      </c>
+      <c r="C27" s="22">
+        <v>135398634</v>
+      </c>
+      <c r="D27" s="20" t="s">
+        <v>1803</v>
+      </c>
+      <c r="E27" s="22">
+        <v>135398634</v>
+      </c>
+      <c r="F27" t="s">
+        <v>1929</v>
+      </c>
+      <c r="G27" t="s">
+        <v>1930</v>
+      </c>
+      <c r="H27" s="24" t="s">
+        <v>1931</v>
+      </c>
+      <c r="I27">
+        <v>135398634</v>
+      </c>
+      <c r="J27" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A28" s="20" t="s">
+        <v>11</v>
+      </c>
+      <c r="B28" s="21" t="s">
+        <v>1843</v>
+      </c>
+      <c r="C28" s="22">
+        <v>277</v>
+      </c>
+      <c r="D28" s="20" t="s">
+        <v>1770</v>
+      </c>
+      <c r="E28" s="22">
+        <v>276</v>
+      </c>
+      <c r="F28" t="s">
+        <v>1932</v>
+      </c>
+      <c r="G28" t="s">
+        <v>1933</v>
+      </c>
+      <c r="H28" s="24" t="s">
+        <v>1934</v>
+      </c>
+      <c r="I28">
+        <v>277</v>
+      </c>
+      <c r="J28" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="B29" s="21" t="s">
+        <v>1804</v>
+      </c>
+      <c r="C29" s="22">
+        <v>43</v>
+      </c>
+      <c r="D29" s="20" t="s">
+        <v>1804</v>
+      </c>
+      <c r="E29" s="22">
+        <v>43</v>
+      </c>
+      <c r="F29" t="s">
+        <v>1935</v>
+      </c>
+      <c r="G29" t="s">
+        <v>1936</v>
+      </c>
+      <c r="H29" s="24" t="s">
+        <v>1937</v>
+      </c>
+      <c r="I29">
+        <v>43</v>
+      </c>
+      <c r="J29" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="B30" s="21" t="s">
+        <v>1844</v>
+      </c>
+      <c r="C30" s="22">
+        <v>1662</v>
+      </c>
+      <c r="D30" s="20" t="s">
+        <v>1805</v>
+      </c>
+      <c r="E30" s="22">
+        <v>1662</v>
+      </c>
+      <c r="F30" t="s">
+        <v>1805</v>
+      </c>
+      <c r="G30" t="s">
+        <v>1938</v>
+      </c>
+      <c r="H30" s="24" t="s">
+        <v>1939</v>
+      </c>
+      <c r="I30">
+        <v>1662</v>
+      </c>
+      <c r="J30" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="20" t="s">
+        <v>34</v>
+      </c>
+      <c r="B31" s="21" t="s">
+        <v>1845</v>
+      </c>
+      <c r="C31" s="22">
+        <v>538669</v>
+      </c>
+      <c r="D31" s="20" t="s">
+        <v>1806</v>
+      </c>
+      <c r="E31" s="22">
+        <v>6442606</v>
+      </c>
+      <c r="F31" t="s">
+        <v>1940</v>
+      </c>
+      <c r="G31" t="s">
+        <v>1941</v>
+      </c>
+      <c r="H31" s="24" t="s">
+        <v>1942</v>
+      </c>
+      <c r="I31">
+        <v>6442606</v>
+      </c>
+      <c r="J31" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" ht="18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="20" t="s">
+        <v>0</v>
+      </c>
+      <c r="B32" s="21" t="s">
+        <v>1846</v>
+      </c>
+      <c r="C32" s="22">
+        <v>1135</v>
+      </c>
+      <c r="D32" s="20" t="s">
+        <v>1807</v>
+      </c>
+      <c r="E32" s="22">
+        <v>1135</v>
+      </c>
+      <c r="F32" t="s">
+        <v>1807</v>
+      </c>
+      <c r="G32" t="s">
+        <v>1943</v>
+      </c>
+      <c r="H32" s="24" t="s">
+        <v>1944</v>
+      </c>
+      <c r="I32">
+        <v>1135</v>
+      </c>
+      <c r="J32" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" ht="18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="20" t="s">
+        <v>35</v>
+      </c>
+      <c r="B33" s="21" t="s">
+        <v>1771</v>
+      </c>
+      <c r="C33" s="22">
+        <v>1935</v>
+      </c>
+      <c r="D33" s="20" t="s">
+        <v>1771</v>
+      </c>
+      <c r="E33" s="22">
+        <v>1935</v>
+      </c>
+      <c r="F33" t="s">
+        <v>1771</v>
+      </c>
+      <c r="G33" t="s">
+        <v>1945</v>
+      </c>
+      <c r="H33" s="24" t="s">
+        <v>1946</v>
+      </c>
+      <c r="I33">
+        <v>1935</v>
+      </c>
+      <c r="J33" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A34" s="20" t="s">
+        <v>6</v>
+      </c>
+      <c r="B34" s="21" t="s">
+        <v>1847</v>
+      </c>
+      <c r="C34" s="22"/>
+      <c r="D34" s="20" t="s">
+        <v>1808</v>
+      </c>
+      <c r="E34" s="22"/>
+      <c r="F34" t="s">
+        <v>1808</v>
+      </c>
+      <c r="G34" t="s">
+        <v>1947</v>
+      </c>
+      <c r="H34" s="24" t="s">
+        <v>1948</v>
+      </c>
+      <c r="I34">
+        <v>129651811</v>
+      </c>
+      <c r="J34" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" ht="18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="B35" s="21" t="s">
+        <v>1848</v>
+      </c>
+      <c r="C35" s="22">
+        <v>119494</v>
+      </c>
+      <c r="D35" s="20" t="s">
+        <v>1809</v>
+      </c>
+      <c r="E35" s="22">
+        <v>119494</v>
+      </c>
+      <c r="F35" t="s">
+        <v>1809</v>
+      </c>
+      <c r="G35" s="16" t="s">
+        <v>1949</v>
+      </c>
+      <c r="H35" s="24" t="s">
+        <v>1950</v>
+      </c>
+      <c r="I35">
+        <v>119494</v>
+      </c>
+      <c r="J35" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" ht="18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="20" t="s">
+        <v>10</v>
+      </c>
+      <c r="B36" s="21" t="s">
+        <v>1849</v>
+      </c>
+      <c r="C36" s="22">
+        <v>6514</v>
+      </c>
+      <c r="D36" s="20" t="s">
+        <v>1786</v>
+      </c>
+      <c r="E36" s="22">
+        <v>6514</v>
+      </c>
+      <c r="F36" t="s">
+        <v>1951</v>
+      </c>
+      <c r="G36" t="s">
+        <v>1952</v>
+      </c>
+      <c r="H36" s="24" t="s">
+        <v>1953</v>
+      </c>
+      <c r="I36">
+        <v>6514</v>
+      </c>
+      <c r="J36" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A37" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="B37" s="21" t="s">
+        <v>1850</v>
+      </c>
+      <c r="C37" s="22">
+        <v>73850</v>
+      </c>
+      <c r="D37" s="20" t="s">
+        <v>1772</v>
+      </c>
+      <c r="E37" s="22">
+        <v>5282713</v>
+      </c>
+      <c r="F37" t="s">
+        <v>1954</v>
+      </c>
+      <c r="G37" t="s">
+        <v>1955</v>
+      </c>
+      <c r="H37" s="24" t="s">
+        <v>1956</v>
+      </c>
+      <c r="I37">
+        <v>73850</v>
+      </c>
+      <c r="J37" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" ht="18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B38" s="9" t="s">
+        <v>1848</v>
+      </c>
+      <c r="C38" s="13">
+        <v>119494</v>
+      </c>
+      <c r="D38" s="5" t="s">
+        <v>1809</v>
+      </c>
+      <c r="E38" s="13">
+        <v>119494</v>
+      </c>
+      <c r="F38" t="s">
+        <v>1809</v>
+      </c>
+      <c r="G38" s="16" t="s">
+        <v>1949</v>
+      </c>
+      <c r="H38" s="24" t="s">
+        <v>1950</v>
+      </c>
+      <c r="I38">
+        <v>119494</v>
+      </c>
+      <c r="J38" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" ht="18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B39" s="9" t="s">
+        <v>1851</v>
+      </c>
+      <c r="C39" s="13">
+        <v>269697</v>
+      </c>
+      <c r="D39" s="5" t="s">
+        <v>1810</v>
+      </c>
+      <c r="E39" s="13">
+        <v>269697</v>
+      </c>
+      <c r="F39" t="s">
+        <v>1957</v>
+      </c>
+      <c r="G39" t="s">
+        <v>1958</v>
+      </c>
+      <c r="H39" s="24" t="s">
+        <v>1959</v>
+      </c>
+      <c r="I39">
+        <v>269697</v>
+      </c>
+      <c r="J39" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A40" s="6" t="s">
+        <v>546</v>
+      </c>
+      <c r="B40" s="10" t="s">
+        <v>1852</v>
+      </c>
+      <c r="C40" s="14"/>
+      <c r="D40" s="6" t="s">
+        <v>1811</v>
+      </c>
+      <c r="E40" s="14">
+        <v>6082</v>
+      </c>
+      <c r="F40" t="s">
+        <v>546</v>
+      </c>
+      <c r="G40" s="23" t="s">
+        <v>1235</v>
+      </c>
+      <c r="H40" s="24" t="s">
+        <v>1960</v>
+      </c>
+      <c r="I40">
+        <v>14345506</v>
+      </c>
+      <c r="J40" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" ht="18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="6" t="s">
+        <v>553</v>
+      </c>
+      <c r="B41" s="10" t="s">
+        <v>1853</v>
+      </c>
+      <c r="C41" s="14"/>
+      <c r="D41" s="6" t="s">
+        <v>1773</v>
+      </c>
+      <c r="E41" s="14"/>
+      <c r="G41" t="s">
+        <v>1961</v>
+      </c>
+      <c r="J41" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A42" s="6" t="s">
+        <v>563</v>
+      </c>
+      <c r="B42" s="10" t="s">
+        <v>1854</v>
+      </c>
+      <c r="C42" s="14"/>
+      <c r="D42" s="6" t="s">
+        <v>1784</v>
+      </c>
+      <c r="E42" s="14"/>
+      <c r="F42" t="s">
+        <v>1854</v>
+      </c>
+      <c r="G42" t="s">
+        <v>1962</v>
+      </c>
+      <c r="H42" s="24" t="s">
+        <v>1963</v>
+      </c>
+      <c r="I42">
+        <v>20606316</v>
+      </c>
+      <c r="J42" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" ht="18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="6" t="s">
+        <v>569</v>
+      </c>
+      <c r="B43" s="10" t="s">
+        <v>1855</v>
+      </c>
+      <c r="C43" s="14">
+        <v>143344</v>
+      </c>
+      <c r="D43" s="6" t="s">
+        <v>1813</v>
+      </c>
+      <c r="E43" s="14">
+        <v>143344</v>
+      </c>
+      <c r="F43" t="s">
+        <v>1813</v>
+      </c>
+      <c r="G43" t="s">
+        <v>1964</v>
+      </c>
+      <c r="H43" s="24" t="s">
+        <v>1965</v>
+      </c>
+      <c r="I43">
+        <v>143344</v>
+      </c>
+      <c r="J43" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" ht="18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="6" t="s">
+        <v>612</v>
+      </c>
+      <c r="B44" s="10" t="s">
+        <v>1817</v>
+      </c>
+      <c r="C44" s="14">
+        <v>4764</v>
+      </c>
+      <c r="D44" s="6" t="s">
+        <v>1817</v>
+      </c>
+      <c r="E44" s="14">
+        <v>4764</v>
+      </c>
+      <c r="F44" t="s">
+        <v>1966</v>
+      </c>
+      <c r="G44" t="s">
+        <v>1967</v>
+      </c>
+      <c r="H44" s="24" t="s">
+        <v>1968</v>
+      </c>
+      <c r="I44">
+        <v>4764</v>
+      </c>
+      <c r="J44" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" ht="18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="6" t="s">
+        <v>622</v>
+      </c>
+      <c r="B45" s="10" t="s">
+        <v>1856</v>
+      </c>
+      <c r="C45" s="14"/>
+      <c r="D45" s="6" t="s">
+        <v>1818</v>
+      </c>
+      <c r="E45" s="14">
+        <v>47955</v>
+      </c>
+      <c r="F45" t="s">
+        <v>1969</v>
+      </c>
+      <c r="G45" t="s">
+        <v>1970</v>
+      </c>
+      <c r="H45" s="24" t="s">
+        <v>1971</v>
+      </c>
+      <c r="I45">
+        <v>47955</v>
+      </c>
+      <c r="J45" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" ht="18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="6" t="s">
+        <v>653</v>
+      </c>
+      <c r="B46" s="10" t="s">
+        <v>1857</v>
+      </c>
+      <c r="C46" s="14">
+        <v>8588</v>
+      </c>
+      <c r="D46" s="6" t="s">
+        <v>1777</v>
+      </c>
+      <c r="E46" s="14">
+        <v>8588</v>
+      </c>
+      <c r="F46" t="s">
+        <v>1972</v>
+      </c>
+      <c r="G46" t="s">
+        <v>1973</v>
+      </c>
+      <c r="H46" s="24" t="s">
+        <v>1974</v>
+      </c>
+      <c r="I46">
+        <v>8588</v>
+      </c>
+      <c r="J46" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" ht="18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="6" t="s">
+        <v>743</v>
+      </c>
+      <c r="B47" s="10" t="s">
+        <v>1858</v>
+      </c>
+      <c r="C47" s="14"/>
+      <c r="D47" s="6" t="s">
+        <v>1819</v>
+      </c>
+      <c r="E47" s="14">
+        <v>9701</v>
+      </c>
+      <c r="F47" t="s">
+        <v>1819</v>
+      </c>
+      <c r="G47" t="s">
+        <v>1975</v>
+      </c>
+      <c r="H47" s="24" t="s">
+        <v>1976</v>
+      </c>
+      <c r="I47">
+        <v>9701</v>
+      </c>
+      <c r="J47" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" ht="18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="6" t="s">
+        <v>746</v>
+      </c>
+      <c r="B48" s="10" t="s">
+        <v>1859</v>
+      </c>
+      <c r="C48" s="14">
+        <v>21236</v>
+      </c>
+      <c r="D48" s="6" t="s">
+        <v>1780</v>
+      </c>
+      <c r="E48" s="14">
+        <v>21236</v>
+      </c>
+      <c r="F48" t="s">
+        <v>288</v>
+      </c>
+      <c r="G48" t="s">
+        <v>1977</v>
+      </c>
+      <c r="H48" s="24" t="s">
+        <v>1978</v>
+      </c>
+      <c r="I48">
+        <v>21236</v>
+      </c>
+      <c r="J48" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A49" s="6" t="s">
+        <v>754</v>
+      </c>
+      <c r="B49" s="10" t="s">
+        <v>1860</v>
+      </c>
+      <c r="C49" s="14">
+        <v>5284604</v>
+      </c>
+      <c r="D49" s="6" t="s">
+        <v>1781</v>
+      </c>
+      <c r="E49" s="14">
+        <v>5284604</v>
+      </c>
+      <c r="F49" t="s">
+        <v>1979</v>
+      </c>
+      <c r="G49" t="s">
+        <v>1980</v>
+      </c>
+      <c r="H49" s="24" t="s">
+        <v>1981</v>
+      </c>
+      <c r="I49">
+        <v>4639</v>
+      </c>
+      <c r="J49" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A50" s="6" t="s">
+        <v>540</v>
+      </c>
+      <c r="B50" s="6"/>
+      <c r="C50" s="6"/>
+      <c r="D50" s="6" t="s">
+        <v>1785</v>
+      </c>
+      <c r="E50" s="6"/>
+      <c r="F50" t="s">
+        <v>1785</v>
+      </c>
+      <c r="G50" t="s">
+        <v>1982</v>
+      </c>
+      <c r="H50" s="24" t="s">
+        <v>1983</v>
+      </c>
+      <c r="I50">
+        <v>14794868</v>
+      </c>
+      <c r="J50" t="b">
+        <f>IF(I50=E50, TRUE, FALSE)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A51" s="6" t="s">
+        <v>549</v>
+      </c>
+      <c r="B51" s="6"/>
+      <c r="C51" s="6"/>
+      <c r="D51" s="6" t="s">
+        <v>1812</v>
+      </c>
+      <c r="E51" s="6"/>
+      <c r="F51" t="s">
+        <v>1812</v>
+      </c>
+      <c r="G51" t="s">
+        <v>1984</v>
+      </c>
+      <c r="H51" s="24" t="s">
+        <v>1985</v>
+      </c>
+      <c r="I51">
+        <v>3406</v>
+      </c>
+      <c r="J51" t="b">
+        <f>IF(I51=E51, TRUE, FALSE)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A52" s="6" t="s">
+        <v>577</v>
+      </c>
+      <c r="B52" s="6"/>
+      <c r="C52" s="6"/>
+      <c r="D52" s="6" t="s">
+        <v>1814</v>
+      </c>
+      <c r="E52" s="6"/>
+      <c r="F52" t="s">
+        <v>1986</v>
+      </c>
+      <c r="G52" t="s">
+        <v>1987</v>
+      </c>
+      <c r="H52" s="24" t="s">
+        <v>1988</v>
+      </c>
+      <c r="I52">
+        <v>6491</v>
+      </c>
+      <c r="J52" t="b">
+        <f>IF(I52=E52, TRUE, FALSE)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A53" s="6" t="s">
+        <v>586</v>
+      </c>
+      <c r="B53" s="6"/>
+      <c r="C53" s="6"/>
+      <c r="D53" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="E53" s="6"/>
+      <c r="F53" t="s">
+        <v>1989</v>
+      </c>
+      <c r="G53" t="s">
+        <v>1990</v>
+      </c>
+      <c r="H53" s="24" t="s">
+        <v>1991</v>
+      </c>
+      <c r="I53">
+        <v>54715757</v>
+      </c>
+      <c r="J53" t="b">
+        <f>IF(I53=E53, TRUE, FALSE)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A54" s="26" t="s">
+        <v>1992</v>
+      </c>
+      <c r="B54" s="6"/>
+      <c r="C54" s="6"/>
+      <c r="D54" s="6" t="s">
+        <v>1815</v>
+      </c>
+      <c r="E54" s="6"/>
+      <c r="F54" t="s">
+        <v>1815</v>
+      </c>
+      <c r="G54" t="s">
+        <v>1993</v>
+      </c>
+      <c r="H54" s="24" t="s">
+        <v>1994</v>
+      </c>
+      <c r="I54">
+        <v>23432</v>
+      </c>
+      <c r="J54" t="b">
+        <f>IF(I54=E54, TRUE, FALSE)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" ht="18" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="6" t="s">
+        <v>604</v>
+      </c>
+      <c r="B55" s="6"/>
+      <c r="C55" s="6"/>
+      <c r="D55" s="6" t="s">
+        <v>1816</v>
+      </c>
+      <c r="E55" s="6"/>
+      <c r="G55" t="s">
+        <v>1995</v>
+      </c>
+      <c r="J55" t="b">
+        <f>IF(I55=E55, TRUE, FALSE)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A56" s="6" t="s">
+        <v>616</v>
+      </c>
+      <c r="B56" s="6"/>
+      <c r="C56" s="6"/>
+      <c r="D56" s="6" t="s">
+        <v>1783</v>
+      </c>
+      <c r="E56" s="6"/>
+      <c r="F56" t="s">
+        <v>376</v>
+      </c>
+      <c r="G56" t="s">
+        <v>1996</v>
+      </c>
+      <c r="H56" s="24" t="s">
+        <v>1997</v>
+      </c>
+      <c r="I56">
+        <v>8655</v>
+      </c>
+      <c r="J56" t="b">
+        <f>IF(I56=E56, TRUE, FALSE)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A57" s="6" t="s">
+        <v>638</v>
+      </c>
+      <c r="B57" s="6"/>
+      <c r="C57" s="6"/>
+      <c r="D57" s="6" t="s">
+        <v>1774</v>
+      </c>
+      <c r="E57" s="6"/>
+      <c r="F57" t="s">
+        <v>1774</v>
+      </c>
+      <c r="G57" t="s">
+        <v>1998</v>
+      </c>
+      <c r="H57" s="24" t="s">
+        <v>1999</v>
+      </c>
+      <c r="I57">
+        <v>78860</v>
+      </c>
+      <c r="J57" t="b">
+        <f>IF(I57=E57, TRUE, FALSE)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A58" s="6" t="s">
+        <v>642</v>
+      </c>
+      <c r="B58" s="6"/>
+      <c r="C58" s="6"/>
+      <c r="D58" s="6" t="s">
+        <v>1775</v>
+      </c>
+      <c r="E58" s="6"/>
+      <c r="F58" t="s">
+        <v>2000</v>
+      </c>
+      <c r="G58" t="s">
+        <v>2001</v>
+      </c>
+      <c r="H58" s="24" t="s">
+        <v>2002</v>
+      </c>
+      <c r="I58">
+        <v>12202</v>
+      </c>
+      <c r="J58" t="b">
+        <f>IF(I58=E58, TRUE, FALSE)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A59" s="6" t="s">
+        <v>643</v>
+      </c>
+      <c r="B59" s="6"/>
+      <c r="C59" s="6"/>
+      <c r="D59" s="6" t="s">
+        <v>1776</v>
+      </c>
+      <c r="E59" s="6"/>
+      <c r="F59" t="s">
+        <v>2003</v>
+      </c>
+      <c r="G59" s="23" t="s">
+        <v>2004</v>
+      </c>
+      <c r="H59" s="24" t="s">
+        <v>2005</v>
+      </c>
+      <c r="I59">
+        <v>564</v>
+      </c>
+      <c r="J59" t="b">
+        <f>IF(I59=E59, TRUE, FALSE)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A60" s="6" t="s">
+        <v>687</v>
+      </c>
+      <c r="B60" s="6"/>
+      <c r="C60" s="6"/>
+      <c r="D60" s="6" t="s">
+        <v>401</v>
+      </c>
+      <c r="E60" s="6"/>
+      <c r="F60" t="s">
+        <v>401</v>
+      </c>
+      <c r="G60" t="s">
+        <v>2006</v>
+      </c>
+      <c r="H60" s="24" t="s">
+        <v>2007</v>
+      </c>
+      <c r="I60">
+        <v>597</v>
+      </c>
+      <c r="J60" t="b">
+        <f>IF(I60=E60, TRUE, FALSE)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A61" s="6" t="s">
+        <v>700</v>
+      </c>
+      <c r="B61" s="6"/>
+      <c r="C61" s="6"/>
+      <c r="D61" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="E61" s="6"/>
+      <c r="F61" t="s">
+        <v>2008</v>
+      </c>
+      <c r="G61" t="s">
+        <v>2009</v>
+      </c>
+      <c r="H61" s="24" t="s">
+        <v>2010</v>
+      </c>
+      <c r="I61">
+        <v>69221</v>
+      </c>
+      <c r="J61" t="b">
+        <f>IF(I61=E61, TRUE, FALSE)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A62" s="6" t="s">
+        <v>706</v>
+      </c>
+      <c r="B62" s="6"/>
+      <c r="C62" s="6"/>
+      <c r="D62" s="6" t="s">
+        <v>1782</v>
+      </c>
+      <c r="E62" s="6"/>
+      <c r="F62" t="s">
+        <v>2011</v>
+      </c>
+      <c r="G62" t="s">
+        <v>2012</v>
+      </c>
+      <c r="H62" s="24" t="s">
+        <v>2013</v>
+      </c>
+      <c r="I62">
+        <v>24781</v>
+      </c>
+      <c r="J62" t="b">
+        <f>IF(I62=E62, TRUE, FALSE)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A63" s="6" t="s">
+        <v>713</v>
+      </c>
+      <c r="B63" s="6"/>
+      <c r="C63" s="6"/>
+      <c r="D63" s="6" t="s">
+        <v>1778</v>
+      </c>
+      <c r="E63" s="6"/>
+      <c r="F63" t="s">
+        <v>2014</v>
+      </c>
+      <c r="G63" t="s">
+        <v>2015</v>
+      </c>
+      <c r="H63" s="24" t="s">
+        <v>2016</v>
+      </c>
+      <c r="I63">
+        <v>3840</v>
+      </c>
+      <c r="J63" t="b">
+        <f>IF(I63=E63, TRUE, FALSE)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A64" s="6" t="s">
+        <v>718</v>
+      </c>
+      <c r="B64" s="6"/>
+      <c r="C64" s="6"/>
+      <c r="D64" s="6" t="s">
+        <v>1779</v>
+      </c>
+      <c r="E64" s="6"/>
+      <c r="F64" t="s">
+        <v>1779</v>
+      </c>
+      <c r="G64" t="s">
+        <v>2017</v>
+      </c>
+      <c r="H64" s="24" t="s">
+        <v>2018</v>
+      </c>
+      <c r="I64">
+        <v>6274</v>
+      </c>
+      <c r="J64" t="b">
+        <f>IF(I64=E64, TRUE, FALSE)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A65" s="6" t="s">
+        <v>765</v>
+      </c>
+      <c r="B65" s="6"/>
+      <c r="C65" s="6"/>
+      <c r="D65" s="6" t="s">
+        <v>1820</v>
+      </c>
+      <c r="E65" s="6"/>
+      <c r="F65" t="s">
+        <v>1820</v>
+      </c>
+      <c r="G65" t="s">
+        <v>2019</v>
+      </c>
+      <c r="H65" s="24" t="s">
+        <v>2020</v>
+      </c>
+      <c r="I65">
+        <v>87</v>
+      </c>
+      <c r="J65" t="b">
+        <f>IF(I65=E65, TRUE, FALSE)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A66" s="6" t="s">
+        <v>766</v>
+      </c>
+      <c r="B66" s="6"/>
+      <c r="C66" s="6"/>
+      <c r="D66" s="6" t="s">
+        <v>767</v>
+      </c>
+      <c r="E66" s="6"/>
+      <c r="F66" t="s">
+        <v>2021</v>
+      </c>
+      <c r="G66" t="s">
+        <v>2022</v>
+      </c>
+      <c r="H66" s="24" t="s">
+        <v>2023</v>
+      </c>
+      <c r="I66">
+        <v>1032</v>
+      </c>
+      <c r="J66" t="b">
+        <f>IF(I66=E66, TRUE, FALSE)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A67" s="6" t="s">
+        <v>780</v>
+      </c>
+      <c r="B67" s="6"/>
+      <c r="C67" s="6"/>
+      <c r="D67" s="6" t="s">
+        <v>1791</v>
+      </c>
+      <c r="E67" s="6"/>
+      <c r="F67" t="s">
+        <v>1824</v>
+      </c>
+      <c r="G67" t="s">
+        <v>2024</v>
+      </c>
+      <c r="H67" s="24" t="s">
+        <v>2025</v>
+      </c>
+      <c r="I67">
+        <v>69980390</v>
+      </c>
+      <c r="J67" t="b">
+        <f>IF(I67=E67, TRUE, FALSE)</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:J67" xr:uid="{2442BCC8-4903-A242-813F-023B53DEA0F4}">
+    <filterColumn colId="9">
       <filters>
         <filter val="FALSE"/>
       </filters>
     </filterColumn>
   </autoFilter>
+  <conditionalFormatting sqref="F1:J1">
+    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
+      <formula>FALSE</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
+      <formula>TRUE</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J1:J1048576">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
+      <formula>FALSE</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <hyperlinks>
+    <hyperlink ref="H9" r:id="rId1" xr:uid="{CE9DE831-FCB4-224E-AA9B-C8CE15493812}"/>
+    <hyperlink ref="H10" r:id="rId2" xr:uid="{FBD18CF5-EEDB-7A47-8462-1E2CC081DF15}"/>
+    <hyperlink ref="H12" r:id="rId3" xr:uid="{55CBE985-4A07-9A43-873A-2538470E1A49}"/>
+    <hyperlink ref="H54" r:id="rId4" xr:uid="{16D8EEDD-4A9E-F74D-A6EA-B57176234EF6}"/>
+    <hyperlink ref="H58" r:id="rId5" xr:uid="{AD11B7D0-2B1F-6E4E-B8BD-2B2AB2478885}"/>
+    <hyperlink ref="H59" r:id="rId6" xr:uid="{A660FEAF-72C3-F34D-843C-D7549F4C5A56}"/>
+    <hyperlink ref="H63" r:id="rId7" xr:uid="{EBF95446-7A06-234B-BDF6-7873803F5A4A}"/>
+    <hyperlink ref="H2" r:id="rId8" xr:uid="{278D4D16-C782-174E-B016-441E93C7BD71}"/>
+    <hyperlink ref="H3" r:id="rId9" xr:uid="{E0CB0A80-FFDD-F04C-B6AE-8DE06B1CC95C}"/>
+    <hyperlink ref="H5" r:id="rId10" xr:uid="{0B84E088-C3BE-1844-A1F9-921F6BF9EE25}"/>
+    <hyperlink ref="H6" r:id="rId11" xr:uid="{9CAE0081-7AD1-E341-B17B-2519E876C0D6}"/>
+    <hyperlink ref="H7" r:id="rId12" xr:uid="{A180844F-23E6-8C4F-9033-3B8B0BD1AE31}"/>
+    <hyperlink ref="H8" r:id="rId13" xr:uid="{9409E609-2F7D-144F-8FB5-5EDD6F785D63}"/>
+    <hyperlink ref="H11" r:id="rId14" xr:uid="{A482D202-9D42-5C45-846A-5E4D66FC4FC9}"/>
+    <hyperlink ref="H13" r:id="rId15" xr:uid="{ED693092-CBB6-6242-9F86-7683E1E31ACC}"/>
+    <hyperlink ref="H16" r:id="rId16" xr:uid="{9A452421-F4AA-D848-A5E5-6D1150F65D3F}"/>
+    <hyperlink ref="H17" r:id="rId17" xr:uid="{11C96BC1-C638-A141-8E84-79C64472AD5D}"/>
+    <hyperlink ref="H19" r:id="rId18" xr:uid="{28A3355F-F34A-A549-A6B9-3081B7151088}"/>
+    <hyperlink ref="H20" r:id="rId19" xr:uid="{4F1D8BBE-6A3E-3E4F-BC25-2FDE2B50AD10}"/>
+    <hyperlink ref="H21" r:id="rId20" xr:uid="{02AFBC4C-B86F-D144-B098-5644F88E6D4A}"/>
+    <hyperlink ref="H22" r:id="rId21" xr:uid="{81D250BB-D371-5544-A44E-CC36AD7027AF}"/>
+    <hyperlink ref="H23" r:id="rId22" xr:uid="{A99D25F6-884F-F748-A468-A4946F152F5E}"/>
+    <hyperlink ref="H25" r:id="rId23" xr:uid="{88340C27-526B-0C47-AF82-1E64DCF9DBA7}"/>
+    <hyperlink ref="H26" r:id="rId24" xr:uid="{678F7C20-FB56-244D-9E97-36462A0DAFD9}"/>
+    <hyperlink ref="H27" r:id="rId25" xr:uid="{BB00C8D5-19D0-8A4B-A426-72BA601D6DD8}"/>
+    <hyperlink ref="H28" r:id="rId26" xr:uid="{6988E323-3914-414C-9015-867E84F70903}"/>
+    <hyperlink ref="H29" r:id="rId27" xr:uid="{1EFBBFEB-C7BE-4B43-AB2B-F22E3F912EB4}"/>
+    <hyperlink ref="H30" r:id="rId28" xr:uid="{B42C8822-9DB0-9444-B57A-42BE62D956B0}"/>
+    <hyperlink ref="H31" r:id="rId29" xr:uid="{F670FE3E-5027-204B-B18B-9FC47E91A2CA}"/>
+    <hyperlink ref="H32" r:id="rId30" xr:uid="{8B47C910-464A-E34E-901E-253319969D98}"/>
+    <hyperlink ref="H33" r:id="rId31" xr:uid="{18E11C71-13D7-124B-A518-593BAF2A8C28}"/>
+    <hyperlink ref="H34" r:id="rId32" xr:uid="{9211BD5B-0246-6147-AB08-A472BB83AB08}"/>
+    <hyperlink ref="H35" r:id="rId33" xr:uid="{4EEB9FB2-2874-1941-BEB8-0EEF139F9320}"/>
+    <hyperlink ref="H36" r:id="rId34" xr:uid="{7C98437C-835F-DA42-A8D6-A23000F11AA2}"/>
+    <hyperlink ref="H37" r:id="rId35" xr:uid="{65F11215-6109-9A4A-B27D-CB6D3712603D}"/>
+    <hyperlink ref="H38" r:id="rId36" xr:uid="{009D3C85-9535-FA40-91CA-5F70594959CB}"/>
+    <hyperlink ref="H39" r:id="rId37" xr:uid="{52B6DE15-2D68-A545-A054-BE7E1B223578}"/>
+    <hyperlink ref="H40" r:id="rId38" xr:uid="{FBAE2621-1036-974F-9626-E2B27612095B}"/>
+    <hyperlink ref="H42" r:id="rId39" xr:uid="{403FF03E-A11C-FC44-B414-0708A91CFD3B}"/>
+    <hyperlink ref="H43" r:id="rId40" xr:uid="{A9E99EC2-79B8-7D4E-83D8-456AC2FDE1ED}"/>
+    <hyperlink ref="H44" r:id="rId41" xr:uid="{07B6EAE3-3419-2142-B3B0-C8ABD8A687CE}"/>
+    <hyperlink ref="H45" r:id="rId42" xr:uid="{2FE61CB4-25A6-A845-87E5-BB3ABDD3F7AA}"/>
+    <hyperlink ref="H46" r:id="rId43" xr:uid="{94ADC617-9C91-C942-BDDF-65DA3C2E00E4}"/>
+    <hyperlink ref="H47" r:id="rId44" xr:uid="{40C44515-E96A-BA40-91FC-6710D700BC40}"/>
+    <hyperlink ref="H48" r:id="rId45" xr:uid="{2143E162-E102-0742-8DBA-96CC79FE049E}"/>
+    <hyperlink ref="H49" r:id="rId46" xr:uid="{B4A10BF3-C5BD-A84E-BFE5-137D56CB125D}"/>
+    <hyperlink ref="H50" r:id="rId47" xr:uid="{78EB001F-75B5-774E-A323-628DEF6823E3}"/>
+    <hyperlink ref="H51" r:id="rId48" xr:uid="{201BEDE3-5987-3A48-9B5C-EB14D24CF998}"/>
+    <hyperlink ref="H52" r:id="rId49" xr:uid="{955C5E68-A110-2D48-AEDD-25206D8640FE}"/>
+    <hyperlink ref="H53" r:id="rId50" xr:uid="{AB8B3010-5069-0447-831F-A3C0812B0489}"/>
+    <hyperlink ref="H56" r:id="rId51" xr:uid="{0B9E368C-BCC4-3449-8F2C-79B916CD66F1}"/>
+    <hyperlink ref="H57" r:id="rId52" xr:uid="{A08BF443-FF3B-9447-A301-641696661AB3}"/>
+    <hyperlink ref="H60" r:id="rId53" xr:uid="{2ACACCB4-344B-F84A-ACAB-BC92297822AA}"/>
+    <hyperlink ref="H61" r:id="rId54" xr:uid="{C36225EE-1C13-4B4B-AA59-6AFDEB5B183E}"/>
+    <hyperlink ref="H62" r:id="rId55" xr:uid="{B5D9686A-4A34-3446-9A0A-EE79A0C93493}"/>
+    <hyperlink ref="H64" r:id="rId56" xr:uid="{4399585A-3A52-2841-8AB6-15814DE21F4A}"/>
+    <hyperlink ref="H65" r:id="rId57" xr:uid="{866B98B8-1A70-764C-B7A4-CD2DCAA31862}"/>
+    <hyperlink ref="H66" r:id="rId58" xr:uid="{7C336761-799D-C74D-AD7F-0A09312BC9B6}"/>
+    <hyperlink ref="H67" r:id="rId59" xr:uid="{AD101C42-97C6-B54A-86CA-6BD6F17A5A62}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>